<commit_message>
feat(profile): implement profile CRUD, PyMuPDF extraction, and master resume lifecycle (Epic 2)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -507,12 +507,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C3" s="18" t="n"/>
-      <c r="D3" s="18" t="n"/>
-      <c r="E3" s="18" t="n"/>
-      <c r="F3" s="18" t="n"/>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="18" t="n"/>
+      <c r="C3" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>3 automated tests passed (API, CRUD, Isolation)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
@@ -669,12 +685,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="18" t="n"/>
+      <c r="C12" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>5 automated tests passed (Unit, API, Security)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
@@ -2697,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3591,6 +3623,446 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-MR-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-MR-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Master_Resume</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PDF Parsing</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PyMuPDF text extraction &amp; section segmentation</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / PyMuPDF</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Valid PDF bytes in-memory</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Synthetic Alice Candidate PDF</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Extract text and call segment_sections</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Text contains all expected sections</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert 'ALICE CANDIDATE' in text and 'skills' in sections</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_pdf_service_text_and_sections</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-MR-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-MR-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Master_Resume</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Skill Detection</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Deterministic tech skill extraction</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / Regex</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Sample text with Python, React, PostgreSQL</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Run detect_skills_deterministically</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Matches known skills with canonical casing; rejects unmentioned skills</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert 'Python' in skills and 'Rust' not in skills</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_pdf_service_deterministic_skill_detection</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-MR-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-MR-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Master_Resume</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>PDF Upload</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Upload master PDF, parse text and auto-seed skills</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Synthetic PDF multipart upload</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>POST /api/v1/resumes</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Returns 201 Created, parses text, auto-populates skills in profile</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 201 and 'Python' in data['extracted_skills']</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_upload_master_resume_pdf</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-MR-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-MR-004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Master_Resume</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Negative Upload</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Reject non-PDF file upload with 400</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>API / Negative</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>malicious.exe binary stream</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>POST /api/v1/resumes with .exe</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Returns 400 Bad Request with descriptive message</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 400 and 'only pdf files' in detail</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_upload_non_pdf_fails</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AUT-MR-005</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TC-MR-005</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Master_Resume</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Negative Upload</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Reject empty 0-byte upload with 400</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>API / Negative</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0-byte PDF stream</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>POST /api/v1/resumes with empty body</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Returns 400 Bad Request</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 400 and 'file is empty' in detail</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_upload_empty_pdf_fails</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10911,7 +11383,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -10999,7 +11470,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11087,7 +11557,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11175,7 +11644,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11263,7 +11731,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11351,7 +11818,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11439,7 +11905,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11527,7 +11992,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11615,7 +12079,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11703,7 +12166,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11791,7 +12253,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -11879,7 +12340,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>Local / Epic-1</t>
@@ -15531,7 +15991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -16425,6 +16885,270 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-PROF-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-PROF-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Profile_Personal</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Profile CRUD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Get and update profile metadata</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>ProfileUpdate payload</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>GET /api/v1/profile, then PUT /api/v1/profile</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Profile auto-initialized, updated with 200 OK</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert updated['headline'] == 'Senior Full-Stack Engineer'</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_get_and_update_profile</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-PROF-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-PROF-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Profile_Personal</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Sub-items CRUD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CRUD for skills, projects, and experiences</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Skill, project, experience payloads</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>POST and DELETE on /profile/skills, /profile/projects, /profile/experiences</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Created with 201, deleted with 204</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert status_code == 201 and delete status == 204</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_profile_subitems_crud</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-PROF-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-PROF-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Profile_Personal</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>User Isolation</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Cross-user profile and resume isolation</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Two distinct registered users</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>User 1 and User 2 tokens</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>User 2 attempts to delete User 1 skill and resume</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Rejected with 404 Not Found; User 2 resume list is empty</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>assert del_skill.status_code == 404 and del_resume.status_code == 404</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_profile_and_resume.py::test_profile_and_resume_user_isolation</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Local / Epic-2</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(jobs): implement Job entity, CRUD endpoints, and Workspace Stage 1 intake (Epic 3)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -719,12 +719,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="18" t="n"/>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="18" t="n"/>
+      <c r="C13" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>5 automated tests passed (API, Validation, Security)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
@@ -3695,7 +3711,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -3783,7 +3798,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -3871,7 +3885,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -3959,7 +3972,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -4047,7 +4059,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -4075,7 +4086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4969,6 +4980,446 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-JOB-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-JOB-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Workspace_Job_Input</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Job Creation</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Create and persist target job record</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>JobCreate payload with TechNova Corp</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Returns 201 Created and persists job record with active status</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 201 and data['company'] == 'TechNova Corp'</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jobs.py::test_create_job_success</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-3</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-JOB-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-JOB-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Workspace_Job_Input</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Enforce non-empty company, title, and JD text</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>API / Negative</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Authenticated candidate</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Payloads with blank title and blank JD</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs with invalid/empty payloads</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Returns 422 Unprocessable Entity</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert r1.status_code == 422 and r2.status_code == 422</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jobs.py::test_create_job_empty_validation</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-3</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-JOB-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-JOB-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Workspace_Job_Input</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Job Retrieval</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>List jobs and retrieve job by ID</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Jobs persisted in DB</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Job IDs</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>GET /api/v1/jobs and GET /api/v1/jobs/{id}</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Returns 200 OK with correct jobs list and job detail</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>assert list_res.status_code == 200 and get_res.json()['company'] == 'Company A'</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jobs.py::test_list_and_get_jobs</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Local / Epic-3</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-JOB-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-JOB-004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Workspace_Job_Input</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Job Mutation</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Update job fields and delete job record</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Existing job in DB</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>JobUpdate payload</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PUT /api/v1/jobs/{id} and DELETE /api/v1/jobs/{id}</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Returns 200 on update, 204 on delete, 404 on subsequent get</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>assert up_res.status_code == 200 and del_res.status_code == 204</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jobs.py::test_update_and_delete_job</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Local / Epic-3</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AUT-JOB-005</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TC-JOB-005</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Workspace_Job_Input</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>User Isolation</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Cross-user job security and isolation</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Two distinct candidates with saved jobs</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>User 1 and User 2 tokens</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET, PUT, DELETE on User 1 job</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Rejected with 404 Not Found; User 2 list is empty</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>assert 404 on all unauthorized access attempts</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jobs.py::test_jobs_user_isolation</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Local / Epic-3</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16957,7 +17408,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -17045,7 +17495,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>
@@ -17133,7 +17582,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Local / Epic-2</t>

</xml_diff>

<commit_message>
feat(analysis): implement Ollama provider, JD requirement extraction, and Workspace Stage 2 (Epic 4)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -753,12 +753,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="18" t="n"/>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="n"/>
+      <c r="C14" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>4 automated tests passed (Unit, API, Security)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
@@ -5052,7 +5068,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-3</t>
@@ -5140,7 +5155,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-3</t>
@@ -5228,7 +5242,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Local / Epic-3</t>
@@ -5316,7 +5329,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>Local / Epic-3</t>
@@ -5404,7 +5416,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Local / Epic-3</t>
@@ -5432,7 +5443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6326,6 +6337,358 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-JDA-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-JDA-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>JD_Analysis</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ollama Abstraction</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Deterministic &amp; local requirement extraction from JD text</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / Provider</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Sample JD text with FastAPI, React, PostgreSQL</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Raw JD string</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Call deterministic_jd_extraction</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Extracts languages, frameworks, tools, cloud, and experience level</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert 'FastAPI' in analysis.frameworks and '5+ Years' in analysis.experience_years</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jd_analysis.py::test_ollama_provider_deterministic_extraction</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-4</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-JDA-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-JDA-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>JD_Analysis</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Trigger Analysis</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Trigger JD analysis and persist JobRequirement record</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Job created in DB</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/analyze</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Execute analysis endpoint and verify persisted response</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Returns 200 OK and structured JobAnalysisResponse</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 200 and 'Python' in data['languages']</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jd_analysis.py::test_analyze_job_and_retrieve_analysis</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-4</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-JDA-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-JDA-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>JD_Analysis</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Validation / Negative</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Reject analysis request for nonexistent job</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>API / Negative</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>job_id=99999</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/99999/analyze</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>assert response.status_code == 404</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jd_analysis.py::test_analyze_nonexistent_job_fails</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Local / Epic-4</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-JDA-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-JDA-004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>JD_Analysis</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Security / Isolation</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Cross-user job analysis access rejection</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Two distinct registered candidates</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>User 1 and User 2 tokens</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET and POST analyze on User 1 job</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found across both operations</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>assert 404 on cross-user analysis access attempts</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_jd_analysis.py::test_job_analysis_user_isolation</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Local / Epic-4</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(matching): implement deterministic matching, evidence alignment, and Workspace Stage 3 (Epic 5)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -787,12 +787,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
+      <c r="C15" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>2 automated tests passed (API, Security)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
@@ -805,12 +821,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
+      <c r="C16" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>2 automated tests passed (Unit, Integrity)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
@@ -6409,7 +6441,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-4</t>
@@ -6497,7 +6528,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-4</t>
@@ -6585,7 +6615,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Local / Epic-4</t>
@@ -6673,7 +6702,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>Local / Epic-4</t>
@@ -6701,7 +6729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7596,6 +7624,182 @@
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-MATCH-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-MATCH-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Match_Analysis</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Deterministic Alignment</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4-category classification &amp; Estimated Job Match scoring</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Profile with Python, FastAPI, and Project</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Job requiring Python, FastAPI, and Kubernetes</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/match</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Classifies into Matched, Weak, Missing, and Unsupported; computes 0-100% score</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert 'Python' in data['matched_skills'] and 'Kubernetes' in data['missing_skills']</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_matching.py::test_match_job_and_retrieve</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-5</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-MATCH-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-MATCH-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Match_Analysis</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Security / Isolation</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Reject cross-user match access</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Two distinct candidates with saved jobs</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>User 1 and User 2 tokens</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET on User 1 match</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert client.get('/jobs/{id}/match', headers=h2).status_code == 404</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_matching.py::test_match_unauthorized_isolation</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-5</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7607,7 +7811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8501,6 +8705,182 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-EVI-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-EVI-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Evidence Drawer</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Link candidate projects &amp; experience to matched skills</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Unit / API</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Profile with projects &amp; experiences</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/match</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Inspect evidence_map in match response</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Every matched skill contains citations to exact project titles</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert any('API Backend Engine' in src for src in data['evidence_map']['Python'])</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_matching.py::test_match_job_and_retrieve</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-5</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-EVI-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-EVI-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Integrity Check</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Detect unsupported claims without project/work backing</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Unit / API</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Skill claimed as Expert with 0 projects</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/match</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Inspect unsupported_claims in response</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Identifies unbacked claims with warning instead of silent approval</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert any('GraphQL' in claim for claim in data['unsupported_claims'])</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_matching.py::test_match_job_and_retrieve</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-5</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(tailoring): implement evidence-grounded tailoring, immutability versioning, Ask AI refinement, and Workspace Stage 4 (Epic 6)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -855,12 +855,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="n"/>
+      <c r="C17" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>Completed (3 automated tests passed)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
@@ -873,12 +889,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
+      <c r="C18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Completed (1 automated test passed)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
@@ -891,12 +923,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
-      <c r="H19" s="18" t="n"/>
+      <c r="C19" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>Completed (2 automated tests passed)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="18" t="inlineStr">
@@ -7695,7 +7743,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-5</t>
@@ -7783,7 +7830,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-5</t>
@@ -8777,7 +8823,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Local / Epic-5</t>
@@ -8865,7 +8910,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Local / Epic-5</t>
@@ -8893,7 +8937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9788,6 +9832,501 @@
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Evidence Grounding</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Draft initial tailored resume from candidate evidence</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API / Integration</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Candidate profile with Python, FastAPI, Docker; Job with Python, FastAPI, Kubernetes</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/tailor</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Generates draft v1 resume populated with real candidate evidence</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>assert res.status_code == 201 and data['version_number'] == 1 and 'summary' in data['content']</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailor_resume_and_non_fabrication</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Non-Fabrication Guardrail</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Ensure missing JD skills are excluded from resume</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Unit / API</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Job JD requires Kubernetes; candidate does NOT possess Kubernetes</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/tailor</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Resume contains Python &amp; FastAPI; strictly does NOT contain Kubernetes</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>assert 'Kubernetes' not in all_skills</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailor_resume_and_non_fabrication</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>User Isolation</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Block cross-user tailoring and version access</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Two distinct users with saved jobs</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET/POST on User 1 tailored resume</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>assert client.get('/tailored-resumes/{id}', headers=u2_headers).status_code == 404</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_security_isolation</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-001</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-001</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Evidence Grounding</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Draft initial tailored resume from candidate evidence</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>API / Integration</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Candidate profile with Python, FastAPI, Docker; Job with Python, FastAPI, Kubernetes</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/tailor</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Generates draft v1 resume populated with real candidate evidence</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>assert res.status_code == 201 and data['version_number'] == 1 and 'summary' in data['content']</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailor_resume_and_non_fabrication</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-002</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-002</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Non-Fabrication Guardrail</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Ensure missing JD skills are excluded from resume</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Unit / API</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Job JD requires Kubernetes; candidate does NOT possess Kubernetes</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>POST /api/v1/jobs/{id}/tailor</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Resume contains Python &amp; FastAPI; strictly does NOT contain Kubernetes</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>assert 'Kubernetes' not in all_skills</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailor_resume_and_non_fabrication</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>AUT-TAILOR-003</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TC-TAILOR-003</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Tailored_Resume</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>User Isolation</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Block cross-user tailoring and version access</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Two distinct users with saved jobs</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET/POST on User 1 tailored resume</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>assert client.get('/tailored-resumes/{id}', headers=u2_headers).status_code == 404</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_security_isolation</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9799,7 +10338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10694,6 +11233,171 @@
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-AIEDIT-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-AIEDIT-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AI_Editing</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Section Refinement</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Request localized AI rewrite with anti-fabrication enforcement</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API / Service</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Tailored draft resume v1</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/tailored-resumes/{id}/edit with section='experience'</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Returns suggested_text, explanation, and factuality_checked=True</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>assert data['factuality_checked'] is True and len(data['suggested_text']) &gt; 10</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_ask_ai_section_editing</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-AIEDIT-001</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-AIEDIT-001</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AI_Editing</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Section Refinement</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Request localized AI rewrite with anti-fabrication enforcement</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>API / Service</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Tailored draft resume v1</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/tailored-resumes/{id}/edit with section='experience'</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Returns suggested_text, explanation, and factuality_checked=True</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>assert data['factuality_checked'] is True and len(data['suggested_text']) &gt; 10</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_ask_ai_section_editing</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10705,7 +11409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11599,6 +12303,336 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-VER-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-VER-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Versioning</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Historical Immutability</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Branch new version when editing or saving snapshot</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Existing draft v1 resume</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>PUT /api/v1/tailored-resumes/{id} with save_as_new_version=True</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Creates v2 resume; v1 remains unchanged</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>assert v2['version_number'] == 2 and v2['parent_version_id'] == v1['id']</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_versioning_and_immutability</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-VER-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-VER-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Versioning</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Final Lock Immutability</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Editing finalized resume forces automatic new version</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Finalized v2 resume</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>PUT /api/v1/tailored-resumes/{id} on finalized resume</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Forces creation of draft v3 instead of mutating locked v2</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>assert v3['version_number'] == 3 and v3['status'] == 'draft'</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_versioning_and_immutability</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-VER-001</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-VER-001</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Versioning</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Historical Immutability</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Branch new version when editing or saving snapshot</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Existing draft v1 resume</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>PUT /api/v1/tailored-resumes/{id} with save_as_new_version=True</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Creates v2 resume; v1 remains unchanged</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>assert v2['version_number'] == 2 and v2['parent_version_id'] == v1['id']</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_versioning_and_immutability</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-VER-002</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-VER-002</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Versioning</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Final Lock Immutability</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Editing finalized resume forces automatic new version</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Finalized v2 resume</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>PUT /api/v1/tailored-resumes/{id} on finalized resume</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Forces creation of draft v3 instead of mutating locked v2</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>assert v3['version_number'] == 3 and v3['status'] == 'draft'</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_tailoring.py::test_tailored_resume_versioning_and_immutability</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Local / Epic-6</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(latex): implement controlled LaTeX injection, pdflatex compiler runner, and Workspace Stage 5 PDF preview (Epic 7)
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -957,12 +957,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
+      <c r="C20" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Completed (4 automated tests passed)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="18" t="inlineStr">
@@ -10144,7 +10160,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -10227,7 +10242,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -10310,7 +10324,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -11381,7 +11394,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -12534,7 +12546,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -12617,7 +12628,6 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
           <t>Local / Epic-6</t>
@@ -14595,7 +14605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15489,6 +15499,338 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-PDF-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-PDF-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PDF_Generation</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>LaTeX Escaping</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sanitize all reserved characters to prevent macro injection and syntax breakage</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Strings containing &amp;, %, $, #, _, {, }, ~, ^, \</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>latex_escape(raw_text)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>All reserved characters properly escaped with TeX control sequences</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>assert r'\&amp;' in escaped and r'\$' in escaped and r'\%' in escaped</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_pdf_generation.py::test_latex_special_character_escaping</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Local / Epic-7</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-PDF-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-PDF-002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PDF_Generation</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Compilation &amp; Persistence</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Invoke pdflatex safely and persist PDF &amp; TeX artifacts</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Integration / API</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Candidate tailored resume draft in DB</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>POST /api/v1/tailored-resumes/{id}/generate-pdf</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Returns 200 with pdf_artifact metadata and positive file size</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>assert data['status'] == 'success' and data['pdf_artifact']['file_size'] &gt; 0</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_pdf_generation.py::test_pdf_compilation_and_artifact_retrieval</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Local / Epic-7</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-PDF-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-PDF-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PDF_Generation</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Document Streaming</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Stream binary PDF and TeX source for preview and download</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Compiled resume PDF and TeX artifacts</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>GET /api/v1/tailored-resumes/{id}/pdf and /tex</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Returns application/pdf and text/plain with proper file content</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>assert stream_res.headers['content-type'] == 'application/pdf'</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_pdf_generation.py::test_pdf_compilation_and_artifact_retrieval</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Local / Epic-7</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-PDF-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-PDF-004</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PDF_Generation</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Security Isolation</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Prevent unauthorized user from accessing or compiling PDF</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest / TestClient</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>User 1 compiled resume artifact</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>User 2 attempts GET on User 1 PDF and artifacts</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Returns 404 Not Found</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>assert client.get('/tailored-resumes/{id}/pdf', headers=u2_headers).status_code == 404</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_pdf_generation.py::test_pdf_generation_user_isolation</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Local / Epic-7</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(epic-9): implement application tracking pipeline and workspace integration
- Add frontend API client `frontend/src/api/applications.js` for CRUD operations and lifecycle status management
- Implement dedicated `ApplicationsPage.jsx` with pipeline status filtering, interview notes editor, and direct PDF download
- Integrate 1-click 'Log Application' action in Workspace Stage 5 linked to target job and tailored resume version
- Record test execution evidence in automation and manual QA workbooks
- Update `PROJECT_STATE.md` marking Epic 9 complete and setting up Epic 10 roadmap
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -17006,7 +17006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17900,6 +17900,354 @@
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
       <c r="R40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AUT-APP-001</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-APP-001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Applications</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Creation &amp; Association</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Create application linked to target job and tailored resume version</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>API / Integration</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Authenticated user with target job &amp; tailored resume</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>POST /api/v1/applications with job_id, tailored_resume_id</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Create application and retrieve list via GET /api/v1/applications</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Application created with 201 status and returned in user list</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>assert res.status_code == 201 and app_data["job_id"] == job_id</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>backend/tests/test_applications.py::test_create_and_list_applications</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Local / Epic-9</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AUT-APP-002</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-APP-001</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Applications</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Status Filter &amp; Transitions</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Filter applications by lifecycle status and update stage notes</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Active tracked application</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/applications/{id} with status=interviewing and notes</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Update status and filter via GET /api/v1/applications?status=interviewing</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Status updated in database and filtered list returns matched records</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>assert update_res.json()["status"] == "interviewing"</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>backend/tests/test_applications.py::test_filter_and_update_application_status</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Local / Epic-9</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AUT-APP-003</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-APP-002</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Applications</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Deletion</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Delete application record safely</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>API / Integration</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Tracked application</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DELETE /api/v1/applications/{id}</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Issue delete request and verify subsequent GET returns 404</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>HTTP 204 No Content returned and record deleted</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>assert del_res.status_code == 204 and get_res.status_code == 404</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>backend/tests/test_applications.py::test_delete_application</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Local / Epic-9</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AUT-APP-004</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-APP-002</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Applications</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Security Isolation</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Prevent unauthorized user from accessing or modifying another candidate's application</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pytest</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>User A application, User B auth token</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GET / PATCH / DELETE /api/v1/applications/{id_a} with User B headers</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>User B attempts read, update, delete, and cross-user job logging</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found preventing cross-tenant access</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>assert status_code == 404 for all cross-user operations</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>backend/tests/test_applications.py::test_application_user_isolation</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Local / Epic-9</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Verified locally</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(epic-10): complete CI testing, security hardening, and E2E verification
</commit_message>
<xml_diff>
--- a/docs/PrivateResume_Automation_Test_Cases.xlsx
+++ b/docs/PrivateResume_Automation_Test_Cases.xlsx
@@ -991,12 +991,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="18" t="n"/>
+      <c r="C21" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Completed (3 automated tests passed: Health, Extractability, Isolation)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
@@ -1009,12 +1025,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="n"/>
+      <c r="C22" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Completed (4 automated tests passed: Creation, Filter, Deletion, Isolation)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
@@ -1027,12 +1059,28 @@
           <t>Automation test-case template</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
+      <c r="C23" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Completed (Security headers middleware &amp; Playwright E2E passed)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>